<commit_message>
perfil-gamer: editable Plano 2026 with available hours, verdict filter on stats top, rename Medíocre to Mediano
</commit_message>
<xml_diff>
--- a/perfil-gamer-src/biblioteca_jogos.xlsx
+++ b/perfil-gamer-src/biblioteca_jogos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estatísticas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biblioteca de Jogos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Estatísticas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Biblioteca de Jogos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -516,14 +516,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -545,8 +545,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -559,10 +559,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -572,10 +572,10 @@
             <idx val="0"/>
             <explosion val="3"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -584,10 +584,10 @@
           <dPt>
             <idx val="1"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -596,10 +596,10 @@
           <dPt>
             <idx val="2"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -609,9 +609,9 @@
             <dLbl>
               <idx val="0"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:uFillTx/>
@@ -632,9 +632,9 @@
             <dLbl>
               <idx val="1"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:uFillTx/>
@@ -655,9 +655,9 @@
             <dLbl>
               <idx val="2"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:uFillTx/>
@@ -676,9 +676,9 @@
               <showPercent val="0"/>
             </dLbl>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -740,16 +740,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -769,10 +769,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -784,14 +784,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -813,8 +813,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -840,10 +840,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="2E5496"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -852,9 +852,9 @@
           <dLbls>
             <numFmt formatCode="General"/>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -970,9 +970,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -994,8 +994,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1006,7 +1006,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1015,9 +1015,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1048,7 +1048,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -1062,7 +1062,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1071,9 +1071,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1097,10 +1097,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1112,14 +1112,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1141,8 +1141,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1168,10 +1168,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1181,10 +1181,10 @@
             <idx val="0"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="1E8449"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1194,10 +1194,10 @@
             <idx val="1"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="27AE60"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1207,10 +1207,10 @@
             <idx val="2"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="52BE80"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1220,10 +1220,10 @@
             <idx val="3"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="A9DFBF"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1233,10 +1233,10 @@
             <idx val="4"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F4D03F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1246,10 +1246,10 @@
             <idx val="5"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F0B27A"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1259,10 +1259,10 @@
             <idx val="6"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="E59866"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1272,10 +1272,10 @@
             <idx val="7"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="CB4335"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1285,10 +1285,10 @@
             <idx val="8"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="922B21"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1299,9 +1299,9 @@
               <idx val="0"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1327,9 +1327,9 @@
               <idx val="1"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1355,9 +1355,9 @@
               <idx val="2"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1383,9 +1383,9 @@
               <idx val="3"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1411,9 +1411,9 @@
               <idx val="4"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,9 +1439,9 @@
               <idx val="5"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1467,9 +1467,9 @@
               <idx val="6"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1495,9 +1495,9 @@
               <idx val="7"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1523,9 +1523,9 @@
               <idx val="8"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1549,9 +1549,9 @@
             </dLbl>
             <numFmt formatCode="General"/>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1661,9 +1661,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1685,8 +1685,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1697,7 +1697,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1706,9 +1706,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1739,7 +1739,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -1751,9 +1751,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1775,8 +1775,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1787,7 +1787,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1796,9 +1796,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1822,10 +1822,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1837,14 +1837,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1866,8 +1866,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1882,10 +1882,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="1A5276"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1894,9 +1894,9 @@
           <dLbls>
             <numFmt formatCode="General"/>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2000,9 +2000,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2024,8 +2024,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2036,7 +2036,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2045,9 +2045,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2078,7 +2078,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2092,7 +2092,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2101,9 +2101,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2127,10 +2127,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2142,14 +2142,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2171,8 +2171,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2187,10 +2187,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="1E8449"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2199,9 +2199,9 @@
           <dLbls>
             <numFmt formatCode="General"/>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2305,9 +2305,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2329,8 +2329,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2341,7 +2341,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2350,9 +2350,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2383,7 +2383,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2397,7 +2397,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2406,9 +2406,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2432,10 +2432,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2447,14 +2447,14 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2476,8 +2476,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2503,10 +2503,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="2E5496"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2514,9 +2514,9 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2586,10 +2586,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="1E8449"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2597,9 +2597,9 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2671,7 +2671,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2680,9 +2680,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2713,7 +2713,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2725,9 +2725,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2749,8 +2749,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2761,7 +2761,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2770,9 +2770,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2796,16 +2796,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2825,10 +2825,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2840,7 +2840,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>7</col>
@@ -2860,9 +2860,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2887,9 +2887,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2914,9 +2914,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2941,9 +2941,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2968,9 +2968,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2995,9 +2995,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+          <c:chart r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3382,6 +3382,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="36">
       <c r="A7" s="43" t="inlineStr">
         <is>
@@ -3389,6 +3390,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="18" customHeight="1" s="36">
       <c r="A9" s="44" t="inlineStr">
         <is>
@@ -3666,6 +3668,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="15" customHeight="1" s="36">
       <c r="A21" s="47" t="inlineStr">
         <is>
@@ -3673,6 +3676,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="18" customHeight="1" s="36">
       <c r="A23" s="48" t="inlineStr">
         <is>
@@ -3930,6 +3934,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35" ht="15" customHeight="1" s="36">
       <c r="A35" s="49" t="inlineStr">
         <is>
@@ -3937,6 +3942,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37" ht="18" customHeight="1" s="36">
       <c r="A37" s="37" t="inlineStr">
         <is>
@@ -4153,6 +4159,7 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="36">
       <c r="A48" s="47" t="inlineStr">
         <is>
@@ -4160,6 +4167,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="18" customHeight="1" s="36">
       <c r="A50" s="48" t="inlineStr">
         <is>
@@ -4480,6 +4488,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="59"/>
     <row r="60" ht="15" customHeight="1" s="36">
       <c r="A60" s="58" t="inlineStr">
         <is>
@@ -4487,6 +4496,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62" ht="18" customHeight="1" s="36">
       <c r="A62" s="59" t="inlineStr">
         <is>
@@ -4595,6 +4605,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72" ht="15" customHeight="1" s="36">
       <c r="A72" s="47" t="inlineStr">
         <is>
@@ -4602,6 +4613,7 @@
         </is>
       </c>
     </row>
+    <row r="73"/>
     <row r="74" ht="18" customHeight="1" s="36">
       <c r="A74" s="48" t="inlineStr">
         <is>
@@ -4908,7 +4920,7 @@
       </c>
       <c r="L3" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M3" s="68" t="inlineStr">
@@ -4957,7 +4969,7 @@
       </c>
       <c r="L4" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M4" s="65" t="inlineStr">
@@ -5325,7 +5337,7 @@
       </c>
       <c r="L12" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M12" s="68" t="inlineStr">
@@ -5509,7 +5521,7 @@
       </c>
       <c r="L16" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M16" s="68" t="n"/>
@@ -5739,7 +5751,7 @@
       </c>
       <c r="L21" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M21" s="68" t="n"/>
@@ -6064,7 +6076,7 @@
       </c>
       <c r="L28" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M28" s="65" t="inlineStr">
@@ -6681,7 +6693,7 @@
       </c>
       <c r="L41" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M41" s="65" t="n"/>
@@ -6730,7 +6742,7 @@
       </c>
       <c r="L42" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M42" s="68" t="n"/>
@@ -6777,7 +6789,7 @@
       </c>
       <c r="L43" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M43" s="65" t="n"/>
@@ -7155,7 +7167,7 @@
       </c>
       <c r="L51" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M51" s="65" t="n"/>
@@ -7404,7 +7416,7 @@
       </c>
       <c r="L56" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M56" s="68" t="n"/>
@@ -7588,7 +7600,7 @@
       </c>
       <c r="L60" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M60" s="68" t="n"/>
@@ -7733,7 +7745,7 @@
       </c>
       <c r="L63" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M63" s="65" t="n"/>

</xml_diff>

<commit_message>
perfil-gamer: editable Plano 2026 with available hours, verdict filter on stats top, rename Medíocre to Mediano (#28)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/perfil-gamer-src/biblioteca_jogos.xlsx
+++ b/perfil-gamer-src/biblioteca_jogos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estatísticas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biblioteca de Jogos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Estatísticas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Biblioteca de Jogos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -516,14 +516,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -545,8 +545,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -559,10 +559,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -572,10 +572,10 @@
             <idx val="0"/>
             <explosion val="3"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -584,10 +584,10 @@
           <dPt>
             <idx val="1"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -596,10 +596,10 @@
           <dPt>
             <idx val="2"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -609,9 +609,9 @@
             <dLbl>
               <idx val="0"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:uFillTx/>
@@ -632,9 +632,9 @@
             <dLbl>
               <idx val="1"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:uFillTx/>
@@ -655,9 +655,9 @@
             <dLbl>
               <idx val="2"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:uFillTx/>
@@ -676,9 +676,9 @@
               <showPercent val="0"/>
             </dLbl>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -740,16 +740,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -769,10 +769,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -784,14 +784,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -813,8 +813,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -840,10 +840,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="2E5496"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -852,9 +852,9 @@
           <dLbls>
             <numFmt formatCode="General"/>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -970,9 +970,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -994,8 +994,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1006,7 +1006,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1015,9 +1015,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1048,7 +1048,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -1062,7 +1062,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1071,9 +1071,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1097,10 +1097,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1112,14 +1112,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1141,8 +1141,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1168,10 +1168,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1181,10 +1181,10 @@
             <idx val="0"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="1E8449"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1194,10 +1194,10 @@
             <idx val="1"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="27AE60"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1207,10 +1207,10 @@
             <idx val="2"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="52BE80"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1220,10 +1220,10 @@
             <idx val="3"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="A9DFBF"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1233,10 +1233,10 @@
             <idx val="4"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F4D03F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1246,10 +1246,10 @@
             <idx val="5"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F0B27A"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1259,10 +1259,10 @@
             <idx val="6"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="E59866"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1272,10 +1272,10 @@
             <idx val="7"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="CB4335"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1285,10 +1285,10 @@
             <idx val="8"/>
             <invertIfNegative val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="922B21"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1299,9 +1299,9 @@
               <idx val="0"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1327,9 +1327,9 @@
               <idx val="1"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1355,9 +1355,9 @@
               <idx val="2"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1383,9 +1383,9 @@
               <idx val="3"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1411,9 +1411,9 @@
               <idx val="4"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,9 +1439,9 @@
               <idx val="5"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1467,9 +1467,9 @@
               <idx val="6"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1495,9 +1495,9 @@
               <idx val="7"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1523,9 +1523,9 @@
               <idx val="8"/>
               <numFmt formatCode="General"/>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1549,9 +1549,9 @@
             </dLbl>
             <numFmt formatCode="General"/>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1661,9 +1661,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1685,8 +1685,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1697,7 +1697,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1706,9 +1706,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1739,7 +1739,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -1751,9 +1751,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1775,8 +1775,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1787,7 +1787,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1796,9 +1796,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1822,10 +1822,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1837,14 +1837,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1866,8 +1866,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1882,10 +1882,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="1A5276"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1894,9 +1894,9 @@
           <dLbls>
             <numFmt formatCode="General"/>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2000,9 +2000,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2024,8 +2024,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2036,7 +2036,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2045,9 +2045,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2078,7 +2078,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2092,7 +2092,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2101,9 +2101,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2127,10 +2127,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2142,14 +2142,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2171,8 +2171,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2187,10 +2187,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="1E8449"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2199,9 +2199,9 @@
           <dLbls>
             <numFmt formatCode="General"/>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2305,9 +2305,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2329,8 +2329,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2341,7 +2341,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2350,9 +2350,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2383,7 +2383,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2397,7 +2397,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2406,9 +2406,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2432,10 +2432,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2447,14 +2447,14 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2476,8 +2476,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2503,10 +2503,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="2E5496"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2514,9 +2514,9 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2586,10 +2586,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="1E8449"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2597,9 +2597,9 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2671,7 +2671,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2680,9 +2680,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2713,7 +2713,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2725,9 +2725,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2749,8 +2749,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2761,7 +2761,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2770,9 +2770,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2796,16 +2796,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr lang="pt-BR" sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2825,10 +2825,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2840,7 +2840,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>7</col>
@@ -2860,9 +2860,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2887,9 +2887,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2914,9 +2914,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2941,9 +2941,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2968,9 +2968,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2995,9 +2995,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+          <c:chart r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3382,6 +3382,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="36">
       <c r="A7" s="43" t="inlineStr">
         <is>
@@ -3389,6 +3390,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="18" customHeight="1" s="36">
       <c r="A9" s="44" t="inlineStr">
         <is>
@@ -3666,6 +3668,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="15" customHeight="1" s="36">
       <c r="A21" s="47" t="inlineStr">
         <is>
@@ -3673,6 +3676,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="18" customHeight="1" s="36">
       <c r="A23" s="48" t="inlineStr">
         <is>
@@ -3930,6 +3934,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35" ht="15" customHeight="1" s="36">
       <c r="A35" s="49" t="inlineStr">
         <is>
@@ -3937,6 +3942,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37" ht="18" customHeight="1" s="36">
       <c r="A37" s="37" t="inlineStr">
         <is>
@@ -4153,6 +4159,7 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="36">
       <c r="A48" s="47" t="inlineStr">
         <is>
@@ -4160,6 +4167,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="18" customHeight="1" s="36">
       <c r="A50" s="48" t="inlineStr">
         <is>
@@ -4480,6 +4488,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="59"/>
     <row r="60" ht="15" customHeight="1" s="36">
       <c r="A60" s="58" t="inlineStr">
         <is>
@@ -4487,6 +4496,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62" ht="18" customHeight="1" s="36">
       <c r="A62" s="59" t="inlineStr">
         <is>
@@ -4595,6 +4605,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72" ht="15" customHeight="1" s="36">
       <c r="A72" s="47" t="inlineStr">
         <is>
@@ -4602,6 +4613,7 @@
         </is>
       </c>
     </row>
+    <row r="73"/>
     <row r="74" ht="18" customHeight="1" s="36">
       <c r="A74" s="48" t="inlineStr">
         <is>
@@ -4908,7 +4920,7 @@
       </c>
       <c r="L3" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M3" s="68" t="inlineStr">
@@ -4957,7 +4969,7 @@
       </c>
       <c r="L4" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M4" s="65" t="inlineStr">
@@ -5325,7 +5337,7 @@
       </c>
       <c r="L12" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M12" s="68" t="inlineStr">
@@ -5509,7 +5521,7 @@
       </c>
       <c r="L16" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M16" s="68" t="n"/>
@@ -5739,7 +5751,7 @@
       </c>
       <c r="L21" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M21" s="68" t="n"/>
@@ -6064,7 +6076,7 @@
       </c>
       <c r="L28" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M28" s="65" t="inlineStr">
@@ -6681,7 +6693,7 @@
       </c>
       <c r="L41" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M41" s="65" t="n"/>
@@ -6730,7 +6742,7 @@
       </c>
       <c r="L42" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M42" s="68" t="n"/>
@@ -6777,7 +6789,7 @@
       </c>
       <c r="L43" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M43" s="65" t="n"/>
@@ -7155,7 +7167,7 @@
       </c>
       <c r="L51" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M51" s="65" t="n"/>
@@ -7404,7 +7416,7 @@
       </c>
       <c r="L56" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M56" s="68" t="n"/>
@@ -7588,7 +7600,7 @@
       </c>
       <c r="L60" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M60" s="68" t="n"/>
@@ -7733,7 +7745,7 @@
       </c>
       <c r="L63" s="62" t="inlineStr">
         <is>
-          <t>Medíocre</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="M63" s="65" t="n"/>

</xml_diff>